<commit_message>
Update Xiaomi TV price list
</commit_message>
<xml_diff>
--- a/Xiaomi电视产品价格表2025-2026.xlsx
+++ b/Xiaomi电视产品价格表2025-2026.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\songmeiyi\Desktop\lab\Amazon_po\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21000" windowHeight="8955"/>
+    <workbookView windowWidth="21195" windowHeight="9487"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="126">
   <si>
     <t>ASIN</t>
   </si>
@@ -329,7 +334,7 @@
     <t>G PRO 27QI 2026</t>
   </si>
   <si>
-    <t>-</t>
+    <t>B0H83QMWSJ</t>
   </si>
   <si>
     <t>G25I 2026</t>
@@ -357,6 +362,54 @@
   </si>
   <si>
     <t>FX Mini LED-75</t>
+  </si>
+  <si>
+    <t>B0H44KWKRS</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F 32</t>
+  </si>
+  <si>
+    <t>B0H448LDSH</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F 43</t>
+  </si>
+  <si>
+    <t>B0H44PLCP3</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F 55</t>
+  </si>
+  <si>
+    <t>B0H44H5QPH</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F 65</t>
+  </si>
+  <si>
+    <t>B0H7BF91XG</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F Pro 32</t>
+  </si>
+  <si>
+    <t>B0H44MW1ST</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F Pro 43</t>
+  </si>
+  <si>
+    <t>B0H448WZ71</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F Pro 55</t>
+  </si>
+  <si>
+    <t>B0H7BBDZTR</t>
+  </si>
+  <si>
+    <t>NEW Xiaomi TV F Pro 65</t>
   </si>
 </sst>
 </file>
@@ -1043,7 +1096,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1078,6 +1131,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1604,7 +1663,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5"/>
   <cols>
     <col min="4" max="4" width="28.0176991150442" style="1" customWidth="1"/>
@@ -2192,7 +2251,7 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="7"/>
-      <c r="B53" t="s">
+      <c r="B53" s="13" t="s">
         <v>100</v>
       </c>
       <c r="C53" s="10"/>
@@ -2231,6 +2290,70 @@
       </c>
       <c r="D57" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="B58" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="B59" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="D59" s="14" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="B60" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="B61" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D61" s="14" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="B62" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D62" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="B63" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D63" s="14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="B64" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D64" s="14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="D65" s="14" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>